<commit_message>
Add FR as the sheet name
</commit_message>
<xml_diff>
--- a/data/FRS_cleaned/Dec/Fmn D Dec/WorkOrderLocal_Dec 2025 D.xlsx
+++ b/data/FRS_cleaned/Dec/Fmn D Dec/WorkOrderLocal_Dec 2025 D.xlsx
@@ -5,23 +5,22 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\fwDemo\data\FRS_cleaned\Dec\Fmn D Dec\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Anu\APT\apt\army\fortwilliam\code\fwDemo\data\FRS_cleaned\Dec\Fmn D Dec\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64993F54-C3CE-4664-A8B3-0E09AC0B57C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68D3211F-D2E2-48D3-A084-55315BC29EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="-15720" windowWidth="28800" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="FR" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="139">
   <si>
     <t>No</t>
   </si>
@@ -36,12 +35,6 @@
   <si>
     <t>DRWO fwd to W1 vide Z1 letter No 70301/DRWO/TC/WKSP dt 31 May 2025.
 Unit directed vide 'U8,U100 letter No 24502/VVksp/Gen dt 07 Jan 2026 to fwd eqpl lo 'US for declaring it BER and further demand.</t>
-  </si>
-  <si>
-    <t>DRWO fwd to W1 vide 'U8 DRWO No FWD/DRWO/A VEH/TECH/12/25 dt 11 Mar 25.</t>
-  </si>
-  <si>
-    <t>Unit directed vide 'US, U100 letter No 24502/Wksp/Gen dt 07 Jan 2026 to fwd eqpt to·ua for declaring it BER and further demand.</t>
   </si>
   <si>
     <t>DRWO fwd to W1 vide 'U8 DRWO No FWD/DRWO/A VEH/TECH/11/25 dt 11 Mar 25. Eaot denosited with W1 for r""air on 17 Mav 25.</t>
@@ -187,21 +180,6 @@
     <t>18X 0119N51</t>
   </si>
   <si>
-    <t>18X 0119N52</t>
-  </si>
-  <si>
-    <t>18X 0119N53</t>
-  </si>
-  <si>
-    <t>18X 0119N54</t>
-  </si>
-  <si>
-    <t>18X 0119N55</t>
-  </si>
-  <si>
-    <t>18X 0119N56</t>
-  </si>
-  <si>
     <t>18X 0119N57</t>
   </si>
   <si>
@@ -844,570 +822,11 @@
     <r>
       <rPr>
         <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Control Unit K1 faulty</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">DRWO </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">fwd </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>W1 vide Z1 letter No 70301/DRWO/TC/WKSP dt 31 May 2025</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF676969"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Unit directed </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>vide 'US</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF3F423F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">U100 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">letter No 24502/Wksp/Gen dt 07 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Jan </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF2F312F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">to fwd eqpt to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF2F312F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>U</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF2F312F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">S </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>for declaring ii BER and further demand</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF525654"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>TKN-4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF2F312F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">S </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">fwd to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>F</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">for </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>upgradation</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Under </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>repair at F1 wef 08 Jan 2022</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF525654"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Completion and collection </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">notice </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>not received</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF525654"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Amplidyne </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">motor </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>faulty</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF2F312F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Cont</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF050505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">rol Unit </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>BV</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF525654"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1A1C1C"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>185</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF525654"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF2F312F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>2S</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1F211F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>TKN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF343A38"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1F211F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>4S fwd t</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF343A38"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">o </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1F211F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>F1 for
-u</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF343A38"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>oo</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1F211F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>radallon</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
         <color rgb="FF1F211F"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
       <t>No</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1F211F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Under repair at F1 wet 06 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF343A38"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Oct </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1F211F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>2022
-Comol</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF343A38"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>etio</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1F211F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">n and collection </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0F110F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">notice not </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1F211F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>r</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF343A38"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>ecei</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1F211F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>ved</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF696E6E"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>.</t>
     </r>
   </si>
   <si>
@@ -3593,11 +3012,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="dd\-mm\-yy;@"/>
-    <numFmt numFmtId="166" formatCode="[$-14009]dd/mm/yyyy;@"/>
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="[$-14009]dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -3660,12 +3078,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF525654"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF676969"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -3762,7 +3174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -3781,19 +3193,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3808,32 +3208,35 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4140,1379 +3543,1274 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACD5C46C-B07C-42BA-9996-0A0B735859A2}">
   <dimension ref="A1:K36"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.33203125" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="12"/>
-    <col min="2" max="2" width="13.5" style="12" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" style="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="12" customWidth="1"/>
-    <col min="5" max="5" width="17.1640625" style="12" customWidth="1"/>
-    <col min="6" max="6" width="18" style="12" customWidth="1"/>
-    <col min="7" max="7" width="14" style="12" customWidth="1"/>
-    <col min="8" max="8" width="30.6640625" style="12" customWidth="1"/>
-    <col min="9" max="9" width="18" style="23" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" style="12" customWidth="1"/>
-    <col min="11" max="11" width="67.83203125" style="12" customWidth="1"/>
-    <col min="12" max="16384" width="9.33203125" style="12"/>
+    <col min="1" max="1" width="9.33203125" style="8"/>
+    <col min="2" max="2" width="13.44140625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" style="8" customWidth="1"/>
+    <col min="6" max="6" width="18" style="8" customWidth="1"/>
+    <col min="7" max="7" width="14" style="8" customWidth="1"/>
+    <col min="8" max="8" width="30.6640625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="18" style="19" customWidth="1"/>
+    <col min="10" max="10" width="12.77734375" style="8" customWidth="1"/>
+    <col min="11" max="11" width="67.77734375" style="8" customWidth="1"/>
+    <col min="12" max="16384" width="9.33203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="H1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:11" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="C2" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="K1" s="1" t="s">
+      <c r="E2" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="51" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>27</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="I2" s="16">
+        <v>84</v>
+      </c>
+      <c r="I2" s="12">
         <v>45377</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="10" t="s">
         <v>0</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13" t="s">
+    <row r="3" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A3" s="20">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" s="13" t="s">
-        <v>47</v>
+      <c r="G3" s="9" t="s">
+        <v>40</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="I3" s="17">
+        <v>85</v>
+      </c>
+      <c r="I3" s="13">
         <v>45057</v>
       </c>
-      <c r="J3" s="8" t="s">
-        <v>93</v>
+      <c r="J3" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>146</v>
+    <row r="4" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>131</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>48</v>
+        <v>27</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>41</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="I4" s="18">
+        <v>87</v>
+      </c>
+      <c r="I4" s="14">
         <v>44810</v>
       </c>
-      <c r="J4" s="8" t="s">
-        <v>93</v>
+      <c r="J4" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="51" x14ac:dyDescent="0.2">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>15</v>
+    <row r="5" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A5" s="20">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="I5" s="16">
+        <v>89</v>
+      </c>
+      <c r="I5" s="12">
         <v>45736</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>97</v>
+      <c r="J5" s="6" t="s">
+        <v>90</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="13"/>
-      <c r="B6" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>146</v>
+    <row r="6" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>131</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="I6" s="14">
+        <v>44816</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="20">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I7" s="12">
+        <v>45743</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="I8" s="15">
+        <v>45936</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A9" s="20">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="I9" s="15">
+        <v>45708</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="I10" s="15">
+        <v>45796</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="20">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I11" s="16">
+        <v>45736</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="I12" s="15">
+        <v>45922</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="20">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="6">
+        <v>13</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="66" x14ac:dyDescent="0.25">
+      <c r="A15" s="20">
+        <v>14</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I15" s="17">
+        <v>45811</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="6">
+        <v>15</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="I16" s="15">
+        <v>45740</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A17" s="20">
+        <v>16</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="I17" s="15">
+        <v>45657</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="A18" s="6">
+        <v>17</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="I18" s="15">
+        <v>45573</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="20">
         <v>18</v>
       </c>
-      <c r="E6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="I6" s="18">
+      <c r="B19" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="I19" s="15">
+        <v>45657</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="6">
+        <v>19</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="I20" s="15">
         <v>44816</v>
       </c>
-      <c r="J6" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>99</v>
+      <c r="J20" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>118</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="I7" s="16">
-        <v>45743</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>101</v>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="20">
+        <v>20</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="I21" s="15">
+        <v>45831</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K21" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="I8" s="19">
-        <v>45936</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>112</v>
+    <row r="22" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A22" s="6">
+        <v>21</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I22" s="15">
+        <v>45353</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="13"/>
-      <c r="B9" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="I9" s="19">
-        <v>45708</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>6</v>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="20">
+        <v>22</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="I23" s="15">
+        <v>45754</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>124</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="51" x14ac:dyDescent="0.2">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" s="3" t="s">
+    <row r="24" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A24" s="6">
+        <v>23</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="I10" s="19">
-        <v>45796</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>7</v>
+      <c r="F24" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I24" s="17">
+        <v>45790</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G11" s="3" t="s">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="20">
+        <v>24</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="I11" s="20">
-        <v>45736</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>116</v>
+      <c r="F25" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="I25" s="15">
+        <v>45916</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G12" s="3" t="s">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="6">
+        <v>25</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H12" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="I12" s="19">
-        <v>45922</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="I13" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A14" s="13"/>
-      <c r="B14" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G14" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="I14" s="18" t="s">
-        <v>123</v>
-      </c>
-      <c r="J14" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="I15" s="21">
-        <v>45811</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="I16" s="19">
-        <v>45740</v>
-      </c>
-      <c r="J16" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K16" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="I17" s="19">
-        <v>45657</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K17" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="51" x14ac:dyDescent="0.2">
-      <c r="A18" s="13"/>
-      <c r="B18" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="I18" s="19">
-        <v>45573</v>
-      </c>
-      <c r="J18" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="I19" s="19">
-        <v>45657</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K19" s="5" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G20" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="I20" s="19">
-        <v>44816</v>
-      </c>
-      <c r="J20" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H21" s="5" t="s">
+      <c r="F26" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H26" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="I21" s="19">
-        <v>45831</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="K21" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G22" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="I22" s="19">
-        <v>45353</v>
-      </c>
-      <c r="J22" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G23" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="I23" s="19">
-        <v>45754</v>
-      </c>
-      <c r="J23" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="13"/>
-      <c r="B24" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D24" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G24" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="I24" s="21">
-        <v>45790</v>
-      </c>
-      <c r="J24" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K24" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G25" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="I25" s="19">
-        <v>45916</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G26" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="I26" s="19">
+      <c r="I26" s="15">
         <v>45950</v>
       </c>
-      <c r="J26" s="8" t="s">
+      <c r="J26" s="6" t="s">
         <v>0</v>
       </c>
       <c r="K26" s="5"/>
     </row>
-    <row r="27" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A27" s="13"/>
-      <c r="B27" s="13" t="s">
+    <row r="27" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A27" s="20">
         <v>26</v>
       </c>
-      <c r="C27" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D27" s="13" t="s">
+      <c r="B27" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="I27" s="15">
+        <v>45903</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="6">
+        <v>27</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="I28" s="15">
+        <v>45923</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K28" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="20">
+        <v>28</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G29" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="H29" s="9"/>
+      <c r="I29" s="18"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="6">
+        <v>29</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="I30" s="15">
+        <v>45831</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K30" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="20">
+        <v>30</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="I31" s="15">
+        <v>45353</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K31" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="6">
+        <v>31</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="I32" s="15">
+        <v>45740</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K32" s="9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="20">
+        <v>32</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="H33" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="I33" s="15">
+        <v>45657</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K33" s="9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="6">
+        <v>33</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="I34" s="15">
+        <v>45831</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K34" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="20">
+        <v>34</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="G35" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="I27" s="19">
-        <v>45903</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K27" s="5" t="s">
-        <v>13</v>
+      <c r="H35" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="I35" s="15">
+        <v>45353</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K35" s="9" t="s">
+        <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A28" s="13"/>
-      <c r="B28" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D28" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G28" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="I28" s="19">
-        <v>45923</v>
-      </c>
-      <c r="J28" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K28" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A29" s="13"/>
-      <c r="B29" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H29" s="13"/>
-      <c r="I29" s="22"/>
-      <c r="J29" s="13"/>
-      <c r="K29" s="13"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G30" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="H30" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="I30" s="19">
-        <v>45831</v>
-      </c>
-      <c r="J30" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K30" s="13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A31" s="13"/>
-      <c r="B31" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D31" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G31" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="H31" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="I31" s="19">
-        <v>45353</v>
-      </c>
-      <c r="J31" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K31" s="13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A32" s="13"/>
-      <c r="B32" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="F32" s="3" t="s">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="6">
+        <v>35</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H36" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G32" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="H32" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="I32" s="19">
-        <v>45740</v>
-      </c>
-      <c r="J32" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K32" s="13" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A33" s="13"/>
-      <c r="B33" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="G33" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="H33" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="I33" s="19">
-        <v>45657</v>
-      </c>
-      <c r="J33" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K33" s="13" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A34" s="13"/>
-      <c r="B34" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D34" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G34" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H34" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="I34" s="19">
-        <v>45831</v>
-      </c>
-      <c r="J34" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K34" s="13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A35" s="13"/>
-      <c r="B35" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D35" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E35" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G35" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H35" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="I35" s="19">
-        <v>45353</v>
-      </c>
-      <c r="J35" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K35" s="13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A36" s="13"/>
-      <c r="B36" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D36" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="G36" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="H36" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="I36" s="19">
+      <c r="I36" s="15">
         <v>45754</v>
       </c>
-      <c r="J36" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K36" s="13" t="s">
-        <v>153</v>
+      <c r="J36" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K36" s="9" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{235E5BAE-4F20-46BB-8547-5995F7837227}">
-  <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:11" s="12" customFormat="1" ht="395.25" x14ac:dyDescent="0.2">
-      <c r="A1" s="13"/>
-      <c r="B1" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="I1" s="6">
-        <v>45796</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" s="12" customFormat="1" ht="153" x14ac:dyDescent="0.2">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G2" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="I2" s="7">
-        <v>44569</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" s="12" customFormat="1" ht="153" x14ac:dyDescent="0.2">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="I3" s="10">
-        <v>45708</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" s="12" customFormat="1" ht="242.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="I4" s="6">
-        <v>45799</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" s="12" customFormat="1" ht="153" x14ac:dyDescent="0.2">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I5" s="9">
-        <v>45936</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>110</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Simplifying app for demo
</commit_message>
<xml_diff>
--- a/data/FRS_cleaned/Dec/Fmn D Dec/WorkOrderLocal_Dec 2025 D.xlsx
+++ b/data/FRS_cleaned/Dec/Fmn D Dec/WorkOrderLocal_Dec 2025 D.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Anu\APT\apt\army\fortwilliam\code\fwDemo\data\FRS_cleaned\Dec\Fmn D Dec\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21E4FD2-D501-4089-951A-86E5BE634CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13F551B-D65F-428F-94BA-3E06D6A0AC4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="-15780" windowWidth="28800" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2616" yWindow="2616" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FR" sheetId="2" r:id="rId1"/>
@@ -2969,9 +2969,6 @@
     <t>Sys/ Sub Sys</t>
   </si>
   <si>
-    <t>Unit</t>
-  </si>
-  <si>
     <t>65 Armd Regt</t>
   </si>
   <si>
@@ -2997,6 +2994,9 @@
   </si>
   <si>
     <t>Category</t>
+  </si>
+  <si>
+    <t>Units</t>
   </si>
 </sst>
 </file>
@@ -3558,13 +3558,13 @@
         <v>127</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>20</v>
@@ -3593,7 +3593,7 @@
         <v>23</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>16</v>
@@ -3628,7 +3628,7 @@
         <v>23</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>16</v>
@@ -3663,7 +3663,7 @@
         <v>23</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>16</v>
@@ -3698,7 +3698,7 @@
         <v>23</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>16</v>
@@ -3733,7 +3733,7 @@
         <v>23</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>16</v>
@@ -3768,7 +3768,7 @@
         <v>23</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>16</v>
@@ -3803,7 +3803,7 @@
         <v>23</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>17</v>
@@ -3838,7 +3838,7 @@
         <v>23</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>17</v>
@@ -3873,7 +3873,7 @@
         <v>23</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>17</v>
@@ -3908,7 +3908,7 @@
         <v>23</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>17</v>
@@ -3943,7 +3943,7 @@
         <v>23</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>17</v>
@@ -3978,7 +3978,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>17</v>
@@ -4013,7 +4013,7 @@
         <v>23</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>17</v>
@@ -4048,7 +4048,7 @@
         <v>23</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>17</v>
@@ -4083,7 +4083,7 @@
         <v>23</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>17</v>
@@ -4118,7 +4118,7 @@
         <v>23</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>17</v>
@@ -4153,7 +4153,7 @@
         <v>23</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>16</v>
@@ -4188,7 +4188,7 @@
         <v>23</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>16</v>
@@ -4223,7 +4223,7 @@
         <v>23</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>16</v>
@@ -4258,7 +4258,7 @@
         <v>23</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>16</v>
@@ -4293,7 +4293,7 @@
         <v>23</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>16</v>
@@ -4328,7 +4328,7 @@
         <v>23</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>16</v>
@@ -4363,7 +4363,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>17</v>
@@ -4398,7 +4398,7 @@
         <v>23</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>17</v>
@@ -4433,7 +4433,7 @@
         <v>23</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>17</v>
@@ -4448,7 +4448,7 @@
         <v>70</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I26" s="15">
         <v>45950</v>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="K26" s="5"/>
     </row>
-    <row r="27" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="20">
         <v>26</v>
       </c>
@@ -4466,7 +4466,7 @@
         <v>23</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>60</v>
@@ -4501,7 +4501,7 @@
         <v>23</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>60</v>
@@ -4536,7 +4536,7 @@
         <v>23</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>61</v>
@@ -4563,7 +4563,7 @@
         <v>23</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>12</v>
@@ -4598,7 +4598,7 @@
         <v>23</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>12</v>
@@ -4633,7 +4633,7 @@
         <v>23</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>79</v>
@@ -4657,7 +4657,7 @@
         <v>94</v>
       </c>
       <c r="K32" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -4668,7 +4668,7 @@
         <v>23</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>79</v>
@@ -4692,7 +4692,7 @@
         <v>94</v>
       </c>
       <c r="K33" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -4703,7 +4703,7 @@
         <v>23</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>16</v>
@@ -4738,7 +4738,7 @@
         <v>23</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D35" s="9" t="s">
         <v>16</v>
@@ -4773,7 +4773,7 @@
         <v>23</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D36" s="9" t="s">
         <v>79</v>
@@ -4797,7 +4797,7 @@
         <v>94</v>
       </c>
       <c r="K36" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Seperated FR and SPARES from Nov and Dev
</commit_message>
<xml_diff>
--- a/data/FRS_cleaned/Dec/Fmn D Dec/WorkOrderLocal_Dec 2025 D.xlsx
+++ b/data/FRS_cleaned/Dec/Fmn D Dec/WorkOrderLocal_Dec 2025 D.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\fwDemo\data\FRS_cleaned\Dec\Fmn D Dec\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B0F607-E3F8-49B6-83F5-385B9F8E3A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0EEDC38-C03F-43E7-A64B-1FBEFF54CCC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="-16170" windowWidth="28785" windowHeight="13335" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="FR" sheetId="2" r:id="rId1"/>
+    <sheet name="SPARES" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="152">
   <si>
     <t>No</t>
   </si>
@@ -3417,7 +3418,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-14009]dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-14009]dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -3612,31 +3613,31 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3943,7 +3944,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACD5C46C-B07C-42BA-9996-0A0B735859A2}">
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="8"/>
@@ -5210,149 +5211,209 @@
         <v>146</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A37" s="3">
-        <v>36</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D37" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="G37" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="I37" s="13">
-        <v>44569</v>
-      </c>
-      <c r="J37" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="K37" s="5" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A38" s="3">
-        <v>37</v>
-      </c>
-      <c r="B38" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E38" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="G38" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="I38" s="14">
-        <v>45708</v>
-      </c>
-      <c r="J38" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="K38" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A39" s="3">
-        <v>38</v>
-      </c>
-      <c r="B39" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D39" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E39" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G39" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="H39" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="I39" s="12">
-        <v>45799</v>
-      </c>
-      <c r="J39" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="K39" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A40" s="3">
-        <v>39</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E40" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="G40" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="H40" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="I40" s="15">
-        <v>45936</v>
-      </c>
-      <c r="J40" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="K40" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC05B2F5-8C68-43FB-BE84-F9AE30C63974}">
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="9.33203125" style="8"/>
+    <col min="2" max="2" width="13.5" style="8" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="17.1640625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="18" style="8" customWidth="1"/>
+    <col min="7" max="7" width="14" style="8" customWidth="1"/>
+    <col min="8" max="8" width="30.6640625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="18" style="19" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="67.83203125" style="8" customWidth="1"/>
+    <col min="12" max="16384" width="9.33203125" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>36</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="I2" s="13">
+        <v>44569</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>37</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="I3" s="14">
+        <v>45708</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>38</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I4" s="12">
+        <v>45799</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <v>39</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="I5" s="15">
+        <v>45936</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>